<commit_message>
Fix requirement gaps found by the bug board, trace logged bugs in the RTM and SRS, correct the activity diagram, and tidy file names.
</commit_message>
<xml_diff>
--- a/1-RE/RTM.xlsx
+++ b/1-RE/RTM.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -462,7 +462,8 @@
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,6 +511,11 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>Logged Defects (Jira)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
@@ -552,6 +558,11 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>Specified</t>
         </is>
       </c>
@@ -594,6 +605,11 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
+          <t>BUGBPS57-1: Catalog filter returns no results when 'Good with Kids' is combined with Species</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
           <t>Specified</t>
         </is>
       </c>
@@ -631,10 +647,15 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>TC-FR003: Valid submission in queue &lt; 5 s; missing field, non-Ready animal and duplicate open application each rejected</t>
+          <t>TC-FR003: Valid submission in queue &lt; 5 s; missing field, non-Ready or removed animal and duplicate open application each rejected</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>BUGBPS57-2: Questionnaire submission fails silently when the animal listing is deleted mid-submission</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Specified</t>
         </is>
@@ -678,6 +699,11 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
+          <t>BUGBPS57-3: Staff can approve an application without completing the background check</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
           <t>Specified</t>
         </is>
       </c>
@@ -715,10 +741,15 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>TC-FR005: Placement fields required; overdue placement flagged; ending placement returns animal to Ready</t>
+          <t>TC-FR005: Placement fields required; end date after start date; overdue placement flagged; ending placement restores previous status</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>BUGBPS57-4: Foster placement end date allows values earlier than the start date</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Specified</t>
         </is>
@@ -762,6 +793,11 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
           <t>Specified</t>
         </is>
       </c>
@@ -803,6 +839,11 @@
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>BUGBPS57-5: Unauthenticated users can view medical-intake records via direct URL</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Specified</t>
         </is>

</xml_diff>